<commit_message>
Actualización de la tabla de factores de conversión a ppa
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/tabla_ppa.xlsx
+++ b/data-raw/xlsx/tabla_ppa.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucao365-my.sharepoint.com/personal/fernando_gallegos_uca_edu_ar/Documents/proyectos/2026-03-11 Bases EU-SILC/datos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fernando_gallegos\Proyectos\odsa.eusilc\data-raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_0C60FDCE8FF92EB262644615A3F6E4803089D917" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E50B5F7-ADB4-451C-B6AE-D6ED28123632}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBE7321-B3C6-4221-AE73-2412FE0B2B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -213,11 +213,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -522,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -583,16 +584,16 @@
         <v>1.1286099999999999</v>
       </c>
       <c r="H2">
-        <v>1.1309499999999999</v>
+        <v>1.1309400000000001</v>
       </c>
       <c r="I2">
-        <v>1.1262300000000001</v>
+        <v>1.12619</v>
       </c>
       <c r="J2">
         <v>1.12287</v>
       </c>
       <c r="K2">
-        <v>1.1297200000000001</v>
+        <v>1.1311899999999999</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -618,16 +619,16 @@
         <v>0.555176</v>
       </c>
       <c r="H3">
-        <v>0.59382900000000005</v>
+        <v>0.59382699999999999</v>
       </c>
       <c r="I3">
-        <v>0.60456299999999996</v>
+        <v>0.604541</v>
       </c>
       <c r="J3">
-        <v>0.61785800000000002</v>
+        <v>0.61785599999999996</v>
       </c>
       <c r="K3">
-        <v>0.63723799999999997</v>
+        <v>0.63745300000000005</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -653,16 +654,16 @@
         <v>19.693200000000001</v>
       </c>
       <c r="H4">
-        <v>20.210699999999999</v>
+        <v>20.210599999999999</v>
       </c>
       <c r="I4">
-        <v>20.134</v>
+        <v>20.133299999999998</v>
       </c>
       <c r="J4">
-        <v>20.444500000000001</v>
+        <v>20.444400000000002</v>
       </c>
       <c r="K4">
-        <v>20.4252</v>
+        <v>20.415600000000001</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -688,16 +689,16 @@
         <v>9.8580900000000007</v>
       </c>
       <c r="H5">
-        <v>9.89072</v>
+        <v>9.8907000000000007</v>
       </c>
       <c r="I5">
-        <v>9.6936599999999995</v>
+        <v>9.6933100000000003</v>
       </c>
       <c r="J5">
-        <v>9.6460600000000003</v>
+        <v>9.6460299999999997</v>
       </c>
       <c r="K5">
-        <v>9.6331199999999999</v>
+        <v>9.6231899999999992</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -726,13 +727,13 @@
         <v>1.1151800000000001</v>
       </c>
       <c r="I6">
-        <v>1.1223700000000001</v>
+        <v>1.12233</v>
       </c>
       <c r="J6">
         <v>1.11741</v>
       </c>
       <c r="K6">
-        <v>1.1167199999999999</v>
+        <v>1.11554</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -758,16 +759,16 @@
         <v>0.83730599999999999</v>
       </c>
       <c r="H7">
-        <v>0.90769</v>
+        <v>0.90768800000000005</v>
       </c>
       <c r="I7">
-        <v>0.91733600000000004</v>
+        <v>0.91730299999999998</v>
       </c>
       <c r="J7">
-        <v>0.918601</v>
+        <v>0.91859900000000005</v>
       </c>
       <c r="K7">
-        <v>0.92223699999999997</v>
+        <v>0.91846499999999998</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -796,13 +797,13 @@
         <v>1.1686399999999999</v>
       </c>
       <c r="I8">
-        <v>1.1852499999999999</v>
+        <v>1.1852100000000001</v>
       </c>
       <c r="J8">
         <v>1.18123</v>
       </c>
       <c r="K8">
-        <v>1.1821200000000001</v>
+        <v>1.17981</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -828,16 +829,16 @@
         <v>0.81647400000000003</v>
       </c>
       <c r="H9">
-        <v>0.814419</v>
+        <v>0.81441699999999995</v>
       </c>
       <c r="I9">
-        <v>0.81109399999999998</v>
+        <v>0.81106400000000001</v>
       </c>
       <c r="J9">
-        <v>0.82121900000000003</v>
+        <v>0.82121699999999997</v>
       </c>
       <c r="K9">
-        <v>0.82764700000000002</v>
+        <v>0.82783099999999998</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -863,16 +864,16 @@
         <v>0.92254199999999997</v>
       </c>
       <c r="H10">
-        <v>0.90595099999999995</v>
+        <v>0.905949</v>
       </c>
       <c r="I10">
-        <v>0.89095000000000002</v>
+        <v>0.89091799999999999</v>
       </c>
       <c r="J10">
-        <v>0.89618600000000004</v>
+        <v>0.89618399999999998</v>
       </c>
       <c r="K10">
-        <v>0.89624400000000004</v>
+        <v>0.89715199999999995</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -901,13 +902,13 @@
         <v>1.1059600000000001</v>
       </c>
       <c r="I11">
-        <v>1.0863</v>
+        <v>1.08626</v>
       </c>
       <c r="J11">
         <v>1.08612</v>
       </c>
       <c r="K11">
-        <v>1.0650200000000001</v>
+        <v>1.0646899999999999</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -933,16 +934,16 @@
         <v>0.63848700000000003</v>
       </c>
       <c r="H12">
-        <v>0.67434799999999995</v>
+        <v>0.674346</v>
       </c>
       <c r="I12">
-        <v>0.68773300000000004</v>
+        <v>0.68770799999999999</v>
       </c>
       <c r="J12">
-        <v>0.71492900000000004</v>
+        <v>0.71492699999999998</v>
       </c>
       <c r="K12">
-        <v>0.73795500000000003</v>
+        <v>0.73975299999999999</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -968,16 +969,16 @@
         <v>0.98036800000000002</v>
       </c>
       <c r="H13">
-        <v>0.95783700000000005</v>
+        <v>0.95783499999999999</v>
       </c>
       <c r="I13">
-        <v>0.96370299999999998</v>
+        <v>0.96366799999999997</v>
       </c>
       <c r="J13">
-        <v>0.95600499999999999</v>
+        <v>0.95600200000000002</v>
       </c>
       <c r="K13">
-        <v>0.95963900000000002</v>
+        <v>0.95887500000000003</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1003,16 +1004,16 @@
         <v>0.91656400000000005</v>
       </c>
       <c r="H14">
-        <v>0.91487099999999999</v>
+        <v>0.91486800000000001</v>
       </c>
       <c r="I14">
-        <v>0.90566899999999995</v>
+        <v>0.905636</v>
       </c>
       <c r="J14">
-        <v>0.904138</v>
+        <v>0.90413600000000005</v>
       </c>
       <c r="K14">
-        <v>0.90153099999999997</v>
+        <v>0.89971500000000004</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1038,16 +1039,16 @@
         <v>0.72758599999999996</v>
       </c>
       <c r="H15">
-        <v>0.76717500000000005</v>
+        <v>0.76717299999999999</v>
       </c>
       <c r="I15">
-        <v>0.78594600000000003</v>
+        <v>0.78591800000000001</v>
       </c>
       <c r="J15">
-        <v>0.791632</v>
+        <v>0.79162900000000003</v>
       </c>
       <c r="K15">
-        <v>0.79274299999999998</v>
+        <v>0.79299799999999998</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1073,16 +1074,16 @@
         <v>0.68971700000000002</v>
       </c>
       <c r="H16">
-        <v>0.75761100000000003</v>
+        <v>0.75760899999999998</v>
       </c>
       <c r="I16">
-        <v>0.78591200000000005</v>
+        <v>0.785883</v>
       </c>
       <c r="J16">
-        <v>0.78288199999999997</v>
+        <v>0.78288000000000002</v>
       </c>
       <c r="K16">
-        <v>0.79710000000000003</v>
+        <v>0.80630000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1108,16 +1109,16 @@
         <v>1.3079700000000001</v>
       </c>
       <c r="H17">
-        <v>1.2954000000000001</v>
+        <v>1.29539</v>
       </c>
       <c r="I17">
-        <v>1.29274</v>
+        <v>1.2926899999999999</v>
       </c>
       <c r="J17">
-        <v>1.3003100000000001</v>
+        <v>1.3003</v>
       </c>
       <c r="K17">
-        <v>1.3115600000000001</v>
+        <v>1.30796</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1143,16 +1144,16 @@
         <v>232.56899999999999</v>
       </c>
       <c r="H18">
-        <v>251.459</v>
+        <v>251.458</v>
       </c>
       <c r="I18">
-        <v>270.70400000000001</v>
+        <v>270.69400000000002</v>
       </c>
       <c r="J18">
-        <v>279.93</v>
+        <v>279.92899999999997</v>
       </c>
       <c r="K18">
-        <v>288.57499999999999</v>
+        <v>288.43700000000001</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1178,16 +1179,16 @@
         <v>0.88820699999999997</v>
       </c>
       <c r="H19">
-        <v>0.90484399999999998</v>
+        <v>0.90484100000000001</v>
       </c>
       <c r="I19">
-        <v>0.90321099999999999</v>
+        <v>0.90317899999999995</v>
       </c>
       <c r="J19">
-        <v>0.92554400000000003</v>
+        <v>0.92554199999999998</v>
       </c>
       <c r="K19">
-        <v>0.92355799999999999</v>
+        <v>0.92249700000000001</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1216,13 +1217,13 @@
         <v>1.1566700000000001</v>
       </c>
       <c r="I20">
-        <v>1.1698200000000001</v>
+        <v>1.16978</v>
       </c>
       <c r="J20">
         <v>1.1661300000000001</v>
       </c>
       <c r="K20">
-        <v>1.1721900000000001</v>
+        <v>1.17334</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1251,13 +1252,13 @@
         <v>1.1137600000000001</v>
       </c>
       <c r="I21">
-        <v>1.1281000000000001</v>
+        <v>1.1280600000000001</v>
       </c>
       <c r="J21">
-        <v>1.1327</v>
+        <v>1.13269</v>
       </c>
       <c r="K21">
-        <v>1.13958</v>
+        <v>1.1396900000000001</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1283,16 +1284,16 @@
         <v>2.7478400000000001</v>
       </c>
       <c r="H22">
-        <v>2.91629</v>
+        <v>2.91628</v>
       </c>
       <c r="I22">
-        <v>3.0746199999999999</v>
+        <v>3.0745100000000001</v>
       </c>
       <c r="J22">
-        <v>3.1080199999999998</v>
+        <v>3.1080100000000002</v>
       </c>
       <c r="K22">
-        <v>3.0919099999999999</v>
+        <v>3.0946099999999999</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1318,16 +1319,16 @@
         <v>0.84729500000000002</v>
       </c>
       <c r="H23">
-        <v>0.83699199999999996</v>
+        <v>0.83699000000000001</v>
       </c>
       <c r="I23">
-        <v>0.82162000000000002</v>
+        <v>0.82159000000000004</v>
       </c>
       <c r="J23">
-        <v>0.82266399999999995</v>
+        <v>0.822662</v>
       </c>
       <c r="K23">
-        <v>0.83918599999999999</v>
+        <v>0.83937300000000004</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1353,16 +1354,16 @@
         <v>2.5905499999999999</v>
       </c>
       <c r="H24">
-        <v>2.80491</v>
+        <v>2.8048999999999999</v>
       </c>
       <c r="I24">
-        <v>2.9057200000000001</v>
+        <v>2.9056199999999999</v>
       </c>
       <c r="J24">
-        <v>2.9997099999999999</v>
+        <v>2.9996999999999998</v>
       </c>
       <c r="K24">
-        <v>3.09301</v>
+        <v>3.1105200000000002</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1388,16 +1389,16 @@
         <v>0.84260000000000002</v>
       </c>
       <c r="H25">
-        <v>0.83381099999999997</v>
+        <v>0.83380900000000002</v>
       </c>
       <c r="I25">
-        <v>0.86122600000000005</v>
+        <v>0.86119500000000004</v>
       </c>
       <c r="J25">
-        <v>0.87761900000000004</v>
+        <v>0.87761699999999998</v>
       </c>
       <c r="K25">
-        <v>0.876888</v>
+        <v>0.877224</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1423,16 +1424,16 @@
         <v>0.76503299999999996</v>
       </c>
       <c r="H26">
-        <v>0.78964100000000004</v>
+        <v>0.78963899999999998</v>
       </c>
       <c r="I26">
-        <v>0.79463899999999998</v>
+        <v>0.79461000000000004</v>
       </c>
       <c r="J26">
-        <v>0.80020000000000002</v>
+        <v>0.80019799999999996</v>
       </c>
       <c r="K26">
-        <v>0.80572100000000002</v>
+        <v>0.80491699999999999</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1461,13 +1462,13 @@
         <v>1.24882</v>
       </c>
       <c r="I27">
-        <v>1.2333000000000001</v>
+        <v>1.23326</v>
       </c>
       <c r="J27">
         <v>1.20204</v>
       </c>
       <c r="K27">
-        <v>1.1826700000000001</v>
+        <v>1.1850099999999999</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1493,16 +1494,16 @@
         <v>13.111800000000001</v>
       </c>
       <c r="H28">
-        <v>13.507099999999999</v>
+        <v>13.507</v>
       </c>
       <c r="I28">
-        <v>13.6349</v>
+        <v>13.634399999999999</v>
       </c>
       <c r="J28">
-        <v>13.5367</v>
+        <v>13.5366</v>
       </c>
       <c r="K28">
-        <v>13.446</v>
+        <v>13.4316</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1531,10 +1532,13 @@
         <v>218.52500000000001</v>
       </c>
       <c r="I29">
-        <v>220.69399999999999</v>
+        <v>220.68600000000001</v>
       </c>
       <c r="J29">
-        <v>226.01</v>
+        <v>226.00899999999999</v>
+      </c>
+      <c r="K29">
+        <v>237.83199999999999</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1560,13 +1564,16 @@
         <v>14.0853</v>
       </c>
       <c r="H30">
-        <v>13.5611</v>
+        <v>13.561</v>
       </c>
       <c r="I30">
-        <v>14.277799999999999</v>
+        <v>14.2773</v>
       </c>
       <c r="J30">
         <v>14.5756</v>
+      </c>
+      <c r="K30">
+        <v>14.8506</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1595,10 +1602,13 @@
         <v>1.5463</v>
       </c>
       <c r="I31">
-        <v>1.5213399999999999</v>
+        <v>1.52128</v>
       </c>
       <c r="J31">
         <v>1.5128200000000001</v>
+      </c>
+      <c r="K31">
+        <v>1.46241</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -1624,16 +1634,19 @@
         <v>1.0486800000000001</v>
       </c>
       <c r="H32">
-        <v>1.02569</v>
+        <v>1.0256799999999999</v>
       </c>
       <c r="I32">
-        <v>1.0577799999999999</v>
+        <v>1.0577399999999999</v>
       </c>
       <c r="J32">
         <v>1.05888</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K32">
+        <v>1.06392</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1659,13 +1672,16 @@
         <v>1.06498</v>
       </c>
       <c r="I33">
-        <v>1.07341</v>
+        <v>1.0733699999999999</v>
       </c>
       <c r="J33">
-        <v>1.07697</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+        <v>1.0769599999999999</v>
+      </c>
+      <c r="K33">
+        <v>1.09616</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -1688,16 +1704,19 @@
         <v>0.521231</v>
       </c>
       <c r="H34">
-        <v>0.55051700000000003</v>
+        <v>0.55051499999999998</v>
       </c>
       <c r="I34">
-        <v>0.56962800000000002</v>
+        <v>0.56960699999999997</v>
       </c>
       <c r="J34">
-        <v>0.57384599999999997</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.57384500000000005</v>
+      </c>
+      <c r="K34">
+        <v>0.58162199999999997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -1720,16 +1739,19 @@
         <v>28.1098</v>
       </c>
       <c r="H35">
-        <v>29.808</v>
+        <v>29.8079</v>
       </c>
       <c r="I35">
-        <v>31.1921</v>
+        <v>31.190999999999999</v>
       </c>
       <c r="J35">
-        <v>31.21</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+        <v>31.209900000000001</v>
+      </c>
+      <c r="K35">
+        <v>32.136600000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -1752,16 +1774,19 @@
         <v>64.534899999999993</v>
       </c>
       <c r="H36">
-        <v>64.161500000000004</v>
+        <v>64.161299999999997</v>
       </c>
       <c r="I36">
-        <v>63.1661</v>
+        <v>63.163800000000002</v>
       </c>
       <c r="J36">
-        <v>63.242899999999999</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+        <v>63.242699999999999</v>
+      </c>
+      <c r="K36">
+        <v>62.818399999999997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -1784,16 +1809,19 @@
         <v>64.445999999999998</v>
       </c>
       <c r="H37">
-        <v>69.361900000000006</v>
+        <v>69.361699999999999</v>
       </c>
       <c r="I37">
-        <v>71.581800000000001</v>
+        <v>71.5792</v>
       </c>
       <c r="J37">
-        <v>71.870800000000003</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+        <v>71.870599999999996</v>
+      </c>
+      <c r="K37">
+        <v>73.528700000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1816,16 +1844,20 @@
         <v>4.31372</v>
       </c>
       <c r="H38">
-        <v>7.3841099999999997</v>
+        <v>7.3840899999999996</v>
       </c>
       <c r="I38">
-        <v>11.8804</v>
+        <v>11.88</v>
       </c>
       <c r="J38">
-        <v>18.2135</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+        <v>18.2134</v>
+      </c>
+      <c r="K38">
+        <v>25.459399999999999</v>
+      </c>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1851,13 +1883,16 @@
         <v>1.61991</v>
       </c>
       <c r="I39">
-        <v>1.60097</v>
+        <v>1.6009100000000001</v>
       </c>
       <c r="J39">
         <v>1.59433</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K39">
+        <v>1.5712200000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -1883,10 +1918,13 @@
         <v>153.76499999999999</v>
       </c>
       <c r="I40">
-        <v>150.22200000000001</v>
+        <v>150.21600000000001</v>
       </c>
       <c r="J40">
-        <v>150.60499999999999</v>
+        <v>150.60400000000001</v>
+      </c>
+      <c r="K40">
+        <v>152.53399999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>